<commit_message>
new partecipant added, results updated
</commit_message>
<xml_diff>
--- a/app/analysis/results.xlsx
+++ b/app/analysis/results.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1246,6 +1246,49 @@
       </c>
       <c r="M18" s="3" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1630,70 +1673,70 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>48</v>
+        <v>45.5</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>8</v>
+        <v>8.23</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>109</v>
+        <v>102.5</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>25.24</v>
+        <v>24.37</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13.33</v>
+        <v>12.5</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>3.21</v>
+        <v>3.11</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>1.67</v>
+        <v>1.75</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>1.53</v>
+        <v>1.26</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>1.73</v>
+        <v>1.5</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>5</v>
+        <v>4.25</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>2</v>
+        <v>2.22</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>6.33</v>
+        <v>5.75</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>1.53</v>
+        <v>1.71</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>0.67</v>
+        <v>0.75</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="T5" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U5" s="3" t="n">
-        <v>3</v>
+        <v>3.16</v>
       </c>
       <c r="V5" s="3" t="n">
-        <v>16.67</v>
+        <v>14.75</v>
       </c>
       <c r="W5" s="3" t="n">
-        <v>3.21</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
aggiunti utenti, creati plot e aggiornati dati
</commit_message>
<xml_diff>
--- a/app/analysis/results.xlsx
+++ b/app/analysis/results.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1289,6 +1289,92 @@
       </c>
       <c r="M19" s="3" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>145</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="M20" s="3" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1527,49 +1613,49 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>53.33</v>
+        <v>54</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>23.69</v>
+        <v>19.39</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>127</v>
+        <v>131.5</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>58.03</v>
+        <v>48.23</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>15.33</v>
+        <v>16</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>7.37</v>
+        <v>6.16</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>1</v>
+        <v>0.82</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>2.33</v>
+        <v>2.5</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>2.08</v>
+        <v>1.73</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>2.67</v>
+        <v>3.75</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>2.52</v>
+        <v>2.99</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
       <c r="Q3" s="3" t="n">
         <v>0.58</v>
@@ -1581,16 +1667,16 @@
         <v>0</v>
       </c>
       <c r="T3" s="3" t="n">
-        <v>14.33</v>
+        <v>13</v>
       </c>
       <c r="U3" s="3" t="n">
-        <v>5.03</v>
+        <v>4.9</v>
       </c>
       <c r="V3" s="3" t="n">
-        <v>11.33</v>
+        <v>12.5</v>
       </c>
       <c r="W3" s="3" t="n">
-        <v>6.66</v>
+        <v>5.92</v>
       </c>
     </row>
     <row r="4">
@@ -1746,25 +1832,25 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>53.33</v>
+        <v>52.5</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>36.95</v>
+        <v>30.22</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>119.33</v>
+        <v>121</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>121.83</v>
+        <v>99.53</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14.67</v>
+        <v>14.75</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>15.01</v>
+        <v>12.26</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.67</v>
+        <v>1</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>1.15</v>
@@ -1773,25 +1859,25 @@
         <v>2</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>3.46</v>
+        <v>2.83</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>5.33</v>
+        <v>4.5</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>9.24</v>
+        <v>7.72</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>2.67</v>
+        <v>2.5</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>4.62</v>
+        <v>3.79</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>0</v>
@@ -1800,16 +1886,16 @@
         <v>0</v>
       </c>
       <c r="T6" s="3" t="n">
-        <v>10.33</v>
+        <v>10.75</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>6.81</v>
+        <v>5.62</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>18</v>
+        <v>16.75</v>
       </c>
       <c r="W6" s="3" t="n">
-        <v>15.59</v>
+        <v>12.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>